<commit_message>
refactor(delaunay): 重构 Bowyer-Watson 网格生成器代码结构
将原有分散的代码模块重构为清晰的功能划分：
- types.py: 定义核心数据结构
- predicates.py: 实现几何谓词
- core.py: 主生成器逻辑
- cavity.py: 空腔操作
- boundary.py: 边界恢复
- utils.py: 辅助函数

删除冗余代码，合并重复实现，代码量减少83%
新增 REFACTORING_SUMMARY.md 记录重构细节
</commit_message>
<xml_diff>
--- a/docs/design/feature_descriptions.xlsx
+++ b/docs/design/feature_descriptions.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19788" windowHeight="13500" activeTab="1"/>
+    <workbookView windowWidth="19830" windowHeight="9135" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="几何" sheetId="1" r:id="rId1"/>
     <sheet name="交互" sheetId="2" r:id="rId2"/>
+    <sheet name="delaunay" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>序号</t>
   </si>
@@ -84,6 +85,13 @@
 4. 取消上一次拾取 ：鼠标右键点击，取消上一次拾取的点
 5. 确认拾取 ：按Enter键确认拾取，点坐标返回到输入框
 6. 创建几何 ：点击"创建"按钮，清除所有黄色高亮点，恢复几何点的红色显示</t>
+  </si>
+  <si>
+    <t>参考 `c:\Users\HighOrderMesh\.vscode\PyMeshGen\delaunay\BOWYER_WATSON_GMSH_DESIGN.md` 对当前项目中的bowyer-watson算法进行检查完善。使单元测试test_bowyer_watson.TestBowyerWatsonJSONConfig.test_anw_bowyer_watson顺利通过，且满足：1.单元数量合理，插入点数合理，使网格尺寸符合尺寸场要求；2.单元质量合理，最小质量应大于0.3；3.边界完整恢复，与原始输入边界保持一致；补充信息：1.运行程序的虚拟环境为conda pymeshgen，2.单元测试使用Unittests；请继续</t>
+  </si>
+  <si>
+    <t>请参考 @delaunay/BOWYER_WATSON_GMSH_DESIGN.md 对 @delaunay/ 下的三角形网格生成算法进行重构优化，使其使单元测试test_bowyer_watson.TestBowyerWatsonJSONConfig.test_anw_bowyer_watson顺利通过，且满足：1.单元数量合理，插入点数合理，使网格尺寸符合尺寸场要求；2.单元质量合理，最小质量应大于0.3；3.边界完整恢复，与原始输入边界保持一致
+  补充信息：1.运行程序的虚拟环境为conda pymeshgen，2.单元测试使用Unittests；</t>
   </si>
 </sst>
 </file>
@@ -1235,9 +1243,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="3" max="3" width="108.222222222222" customWidth="1"/>
+    <col min="3" max="3" width="108.225" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1258,11 +1266,11 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="43.2" spans="1:3">
+    <row r="3" ht="40.5" spans="1:3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1283,62 +1291,87 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="13.5" outlineLevelRow="4" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="7.22222222222222" customWidth="1"/>
-    <col min="2" max="2" width="13.1111111111111" customWidth="1"/>
-    <col min="3" max="3" width="80.7777777777778" customWidth="1"/>
-    <col min="5" max="5" width="41.1111111111111" customWidth="1"/>
-    <col min="7" max="7" width="66.4444444444444" customWidth="1"/>
+    <col min="1" max="1" width="7.225" customWidth="1"/>
+    <col min="2" max="2" width="13.1083333333333" customWidth="1"/>
+    <col min="3" max="3" width="80.775" customWidth="1"/>
+    <col min="5" max="5" width="41.1083333333333" customWidth="1"/>
+    <col min="7" max="7" width="66.4416666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="57.6" spans="1:3">
-      <c r="A2" s="1">
+    <row r="2" ht="54" spans="1:3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" ht="28.8" spans="1:3">
-      <c r="A3" s="1">
+    <row r="3" ht="27" spans="1:3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="57.6" spans="3:3">
-      <c r="C4" s="1" t="s">
+    <row r="4" ht="54" spans="3:3">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" ht="286" customHeight="1" spans="3:7">
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1" outlineLevelCol="1"/>
+  <cols>
+    <col min="2" max="2" width="72.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="144" customHeight="1" spans="2:2">
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" ht="148" customHeight="1" spans="2:2">
+      <c r="B2" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>